<commit_message>
Update: content_projects.xlsx [2026-04-14 18:53 UTC]
</commit_message>
<xml_diff>
--- a/content_projects.xlsx
+++ b/content_projects.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="projects" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="projects" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="settings" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -603,7 +603,11 @@
           <t>Program Partnership</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
           <t>Obligatory sponsor deliverable</t>
@@ -619,7 +623,11 @@
           <t>Client + RTL</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N2" t="inlineStr">
         <is>
           <t>Program Partner</t>
@@ -671,13 +679,21 @@
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="Z2" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AB2" t="n">
         <v>0</v>
       </c>
@@ -746,7 +762,11 @@
           <t>RTL</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N3" t="inlineStr">
         <is>
           <t>Program Partner</t>
@@ -798,13 +818,21 @@
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="Z3" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AB3" t="n">
         <v>0</v>
       </c>
@@ -853,7 +881,11 @@
           <t>Program Partnership</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
           <t>Obligatory sponsor deliverable</t>
@@ -869,7 +901,11 @@
           <t>Client + RTL</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N4" t="inlineStr">
         <is>
           <t>Program Partner</t>
@@ -921,7 +957,11 @@
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="Z4" t="inlineStr">
         <is>
           <t>2026-09-01</t>
@@ -980,7 +1020,11 @@
           <t>Program Partnership</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
           <t>Obligatory sponsor deliverable</t>
@@ -996,7 +1040,11 @@
           <t>Conference Speakers</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N5" t="inlineStr">
         <is>
           <t>Program Partner</t>
@@ -1048,7 +1096,11 @@
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="Z5" t="inlineStr">
         <is>
           <t>2026-09-21</t>
@@ -1127,7 +1179,11 @@
           <t>Conference Speakers</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N6" t="inlineStr">
         <is>
           <t>Program Partner</t>
@@ -1179,13 +1235,21 @@
           <t>2026-04-30</t>
         </is>
       </c>
-      <c r="Y6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="Z6" t="inlineStr">
         <is>
           <t>2026-05-04</t>
         </is>
       </c>
-      <c r="AA6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AB6" t="n">
         <v>0</v>
       </c>
@@ -1234,7 +1298,11 @@
           <t>Commissioned Research</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr">
         <is>
           <t>Obligatory sponsor deliverable</t>
@@ -1250,33 +1318,77 @@
           <t>RTL</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N7" t="inlineStr">
         <is>
           <t>Commissioned Research</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="P7" t="n">
         <v>8135</v>
       </c>
       <c r="Q7" t="n">
         <v>0</v>
       </c>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr"/>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
-      <c r="Y7" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="Z7" t="inlineStr">
         <is>
           <t>2026-12-12</t>
         </is>
       </c>
-      <c r="AA7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AB7" t="n">
         <v>0</v>
       </c>
@@ -1325,7 +1437,11 @@
           <t>Program Partnership</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
           <t>Obligatory sponsor deliverable</t>
@@ -1341,7 +1457,11 @@
           <t>Client + RTL</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N8" t="inlineStr">
         <is>
           <t>Program Partner</t>
@@ -1393,7 +1513,11 @@
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="Y8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="Z8" t="inlineStr">
         <is>
           <t>2026-09-01</t>
@@ -1452,7 +1576,11 @@
           <t>Program Partnership</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
           <t>Obligatory sponsor deliverable</t>
@@ -1468,7 +1596,11 @@
           <t>Client + RTL</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N9" t="inlineStr">
         <is>
           <t>Program Partner</t>
@@ -1520,13 +1652,21 @@
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="Y9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="Z9" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="AA9" t="inlineStr"/>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AB9" t="n">
         <v>0</v>
       </c>
@@ -1538,16 +1678,16 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>White Paper MVRDV NEXT</t>
+          <t>Global Activity Series: Americas (Q1)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>White paper</t>
+          <t>Data study</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1557,12 +1697,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>905a</t>
+          <t>906a</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>WM</t>
+          <t>IW</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1575,23 +1715,31 @@
           <t>Program Partnership</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Obligatory sponsor deliverable</t>
+          <t>Project completed</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Digital</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Client + RTL</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr"/>
+          <t>RTL</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N10" t="inlineStr">
         <is>
           <t>Program Partner</t>
@@ -1599,78 +1747,86 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>MVRDV NEXT (in-kind)</t>
+          <t>Sobha</t>
         </is>
       </c>
       <c r="P10" t="n">
-        <v>0</v>
+        <v>11005</v>
       </c>
       <c r="Q10" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="V10" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-03-09</t>
         </is>
       </c>
       <c r="W10" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="X10" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
-        </is>
-      </c>
-      <c r="Y10" t="inlineStr"/>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="AA10" t="inlineStr"/>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AB10" t="n">
         <v>0</v>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Confirmed</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Global Activity Series: Americas (Q1)</t>
+          <t>Vertical Urbanism Index Report</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Data study</t>
+          <t>PDF report</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1680,7 +1836,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>906a</t>
+          <t>904a</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1698,7 +1854,11 @@
           <t>Program Partnership</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
           <t>Project completed</t>
@@ -1714,7 +1874,11 @@
           <t>RTL</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N11" t="inlineStr">
         <is>
           <t>Program Partner</t>
@@ -1722,57 +1886,65 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Sobha</t>
+          <t>FG | Talls</t>
         </is>
       </c>
       <c r="P11" t="n">
-        <v>11005</v>
+        <v>22875</v>
       </c>
       <c r="Q11" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2025-12-24</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2026-01-08</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="V11" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-01-14</t>
         </is>
       </c>
       <c r="X11" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
-        </is>
-      </c>
-      <c r="Y11" t="inlineStr"/>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
-        </is>
-      </c>
-      <c r="AA11" t="inlineStr"/>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AB11" t="n">
         <v>0</v>
       </c>
@@ -1784,16 +1956,16 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Vertical Urbanism Index Report</t>
+          <t>Global Trends and Forecasts 2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>PDF report</t>
+          <t>Data study</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1803,7 +1975,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>904a</t>
+          <t>906a</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1821,7 +1993,11 @@
           <t>Program Partnership</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J12" t="inlineStr">
         <is>
           <t>Project completed</t>
@@ -1837,7 +2013,11 @@
           <t>RTL</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr"/>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N12" t="inlineStr">
         <is>
           <t>Program Partner</t>
@@ -1845,57 +2025,65 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>FG | Talls</t>
+          <t>Sobha</t>
         </is>
       </c>
       <c r="P12" t="n">
-        <v>22875</v>
+        <v>14531.25</v>
       </c>
       <c r="Q12" t="n">
-        <v>0</v>
+        <v>105</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>2025-12-24</t>
+          <t>2026-01-05</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>2026-01-08</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-01-20</t>
         </is>
       </c>
       <c r="V12" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2026-01-22</t>
         </is>
       </c>
       <c r="W12" t="inlineStr">
         <is>
-          <t>2026-01-14</t>
+          <t>2026-01-29</t>
         </is>
       </c>
       <c r="X12" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
-        </is>
-      </c>
-      <c r="Y12" t="inlineStr"/>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="Z12" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
-        </is>
-      </c>
-      <c r="AA12" t="inlineStr"/>
+          <t>2026-02-06</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AB12" t="n">
         <v>0</v>
       </c>
@@ -1907,31 +2095,31 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Global Trends and Forecasts 2026</t>
+          <t>Vertical Urbanism 6: Q1 2026</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Data study</t>
+          <t>Magazine</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Program Partnership</t>
+          <t>Advertising and Sales-Driven</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>906a</t>
+          <t>701</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>IW</t>
+          <t>DS</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1941,10 +2129,14 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Program Partnership</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr"/>
+          <t>VU Advert</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J13" t="inlineStr">
         <is>
           <t>Project completed</t>
@@ -1957,68 +2149,80 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>RTL</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr"/>
+          <t>External Contributors</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Program Partner</t>
+          <t>Conference Sponsor</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Sobha</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="P13" t="n">
-        <v>14531.25</v>
+        <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2025-11-02</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2025-11-09</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2026-01-12</t>
+          <t>2025-11-16</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2025-11-30</t>
         </is>
       </c>
       <c r="V13" t="inlineStr">
         <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
           <t>2026-01-22</t>
         </is>
       </c>
-      <c r="W13" t="inlineStr">
-        <is>
-          <t>2026-01-29</t>
-        </is>
-      </c>
-      <c r="X13" t="inlineStr">
-        <is>
-          <t>2026-01-30</t>
-        </is>
-      </c>
-      <c r="Y13" t="inlineStr"/>
-      <c r="Z13" t="inlineStr">
-        <is>
-          <t>2026-02-06</t>
-        </is>
-      </c>
-      <c r="AA13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AB13" t="n">
         <v>0</v>
       </c>
@@ -2030,44 +2234,48 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Vertical Urbanism 6: Q1 2026</t>
+          <t>RTL Capacities Brochure</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Magazine</t>
+          <t>PDF report</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Advertising and Sales-Driven</t>
+          <t>Commissioned Research</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>701</t>
+          <t>916</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>DS</t>
+          <t>RD</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>VU Advert</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr"/>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J14" t="inlineStr">
         <is>
           <t>Project completed</t>
@@ -2080,64 +2288,80 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>External Contributors</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr"/>
+          <t>RTL</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N14" t="inlineStr">
         <is>
           <t>Conference Sponsor</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr"/>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="P14" t="n">
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>95</v>
+        <v>150</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>2025-11-02</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>2025-11-09</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>2025-11-16</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>2025-11-30</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>2025-12-01</t>
+          <t>2026-02-18</t>
         </is>
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>2025-12-08</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="X14" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
-        </is>
-      </c>
-      <c r="Y14" t="inlineStr"/>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>2026-01-22</t>
-        </is>
-      </c>
-      <c r="AA14" t="inlineStr"/>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AB14" t="n">
         <v>0</v>
       </c>
@@ -2149,43 +2373,51 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>RTL Capacities Brochure</t>
+          <t>Global Activity Series: Europe (Q2)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>PDF report</t>
+          <t>Data study</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Commissioned Research</t>
+          <t>Program Partnership</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>916</t>
+          <t>906a</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>RD</t>
+          <t>IW</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Program Partnership</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Project completed</t>
+          <t>Obligatory sponsor deliverable</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -2198,61 +2430,77 @@
           <t>RTL</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Conference Sponsor</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr"/>
+          <t>Program Partner</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Sobha</t>
+        </is>
+      </c>
       <c r="P15" t="n">
-        <v>0</v>
+        <v>10385</v>
       </c>
       <c r="Q15" t="n">
-        <v>150</v>
+        <v>75</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>2026-02-18</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
         <is>
-          <t>2026-02-20</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="X15" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
-        </is>
-      </c>
-      <c r="Y15" t="inlineStr"/>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-      <c r="AA15" t="inlineStr"/>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AB15" t="n">
         <v>0</v>
       </c>
@@ -2264,11 +2512,11 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Global Activity Series: Europe (Q2)</t>
+          <t>Global Activity Series: Middle East (Q3)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2301,7 +2549,11 @@
           <t>Program Partnership</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J16" t="inlineStr">
         <is>
           <t>Obligatory sponsor deliverable</t>
@@ -2317,7 +2569,11 @@
           <t>RTL</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N16" t="inlineStr">
         <is>
           <t>Program Partner</t>
@@ -2336,46 +2592,54 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="X16" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="Y16" t="inlineStr"/>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="AA16" t="inlineStr"/>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AB16" t="n">
         <v>0</v>
       </c>
@@ -2387,11 +2651,11 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Global Activity Series: Middle East (Q3)</t>
+          <t>Global Activity Series: Asia (Q4)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2424,7 +2688,11 @@
           <t>Program Partnership</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J17" t="inlineStr">
         <is>
           <t>Obligatory sponsor deliverable</t>
@@ -2440,7 +2708,11 @@
           <t>RTL</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N17" t="inlineStr">
         <is>
           <t>Program Partner</t>
@@ -2459,46 +2731,54 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-11-02</t>
         </is>
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-11-13</t>
         </is>
       </c>
       <c r="X17" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="Y17" t="inlineStr"/>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
-        </is>
-      </c>
-      <c r="AA17" t="inlineStr"/>
+          <t>2026-12-07</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AB17" t="n">
         <v>0</v>
       </c>
@@ -2510,11 +2790,11 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Global Activity Series: Asia (Q4)</t>
+          <t>Sustainability Database and Dashboard</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2529,28 +2809,32 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>906a</t>
+          <t>905a</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>IW</t>
+          <t>WM</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Program Partnership</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr"/>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Obligatory sponsor deliverable</t>
+          <t>Internal commitment</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -2560,10 +2844,14 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>RTL</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr"/>
+          <t>Client + RTL</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N18" t="inlineStr">
         <is>
           <t>Program Partner</t>
@@ -2571,57 +2859,65 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Sobha</t>
+          <t>MVRDV NEXT (in-kind)</t>
         </is>
       </c>
       <c r="P18" t="n">
-        <v>10385</v>
+        <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>75</v>
+        <v>200</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-04-14</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>2026-11-02</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="V18" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>2026-11-13</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="X18" t="inlineStr">
         <is>
-          <t>2026-11-20</t>
-        </is>
-      </c>
-      <c r="Y18" t="inlineStr"/>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>2026-12-07</t>
-        </is>
-      </c>
-      <c r="AA18" t="inlineStr"/>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AB18" t="n">
         <v>0</v>
       </c>
@@ -2633,31 +2929,31 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Sustainability Database and Dashboard</t>
+          <t>Tall + Urban v9</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Data study</t>
+          <t>Book</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Program Partnership</t>
+          <t>Advertising and Sales-Driven</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>905a</t>
+          <t>702</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>WM</t>
+          <t>SU</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2665,8 +2961,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J19" t="inlineStr">
         <is>
           <t>Internal commitment</t>
@@ -2674,73 +2978,85 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Digital</t>
+          <t>Print</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Client + RTL</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr"/>
+          <t>External Contributors</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Program Partner</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>MVRDV NEXT (in-kind)</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="P19" t="n">
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>200</v>
+        <v>307</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="X19" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="Y19" t="inlineStr"/>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
-        </is>
-      </c>
-      <c r="AA19" t="inlineStr"/>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AB19" t="n">
         <v>0</v>
       </c>
@@ -2752,16 +3068,16 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Tall + Urban v9</t>
+          <t>Vertical Urbanism 7: Q2 2026</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Book</t>
+          <t>Magazine</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2771,21 +3087,29 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>702</t>
+          <t>701</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>SU</t>
+          <t>DS</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>VU Advert</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J20" t="inlineStr">
         <is>
           <t>Internal commitment</t>
@@ -2793,7 +3117,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Print</t>
+          <t>Digital</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
@@ -2801,61 +3125,77 @@
           <t>External Contributors</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N20" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr"/>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="P20" t="n">
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>307</v>
+        <v>95</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-03-23</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="Z20" t="inlineStr"/>
-      <c r="AA20" t="inlineStr"/>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="Z20" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AB20" t="n">
         <v>0</v>
       </c>
@@ -2867,11 +3207,11 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Vertical Urbanism 7: Q2 2026</t>
+          <t>Vertical Urbanism 8: Q3 2026</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2904,7 +3244,11 @@
           <t>VU Advert</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J21" t="inlineStr">
         <is>
           <t>Internal commitment</t>
@@ -2912,7 +3256,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Digital</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -2920,13 +3264,21 @@
           <t>External Contributors</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr"/>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N21" t="inlineStr">
         <is>
           <t>Sales</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="P21" t="n">
         <v>0</v>
       </c>
@@ -2935,46 +3287,54 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>2026-03-23</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
-        </is>
-      </c>
-      <c r="Y21" t="inlineStr"/>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
       <c r="Z21" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="AA21" t="inlineStr"/>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AB21" t="n">
         <v>0</v>
       </c>
@@ -2986,31 +3346,31 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Vertical Urbanism 8: Q3 2026</t>
+          <t>Wind Engineering of High-Rise Buildings</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Magazine</t>
+          <t>Book</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Advertising and Sales-Driven</t>
+          <t>Committee-Driven</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>701</t>
+          <t>916</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>DS</t>
+          <t>RD</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -3020,76 +3380,88 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>VU Advert</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr"/>
+          <t>Commissioned Research</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Internal commitment</t>
+          <t>Internal idea</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>External Contributors</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr"/>
+          <t>Committee</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Wind Engineering Cmte</t>
+        </is>
+      </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Sales</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr"/>
+          <t>Commissioned Research</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="P22" t="n">
+        <v>40000</v>
+      </c>
+      <c r="Q22" t="n">
         <v>0</v>
       </c>
-      <c r="Q22" t="n">
-        <v>95</v>
-      </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="Z22" t="inlineStr">
@@ -3097,7 +3469,11 @@
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="AA22" t="inlineStr"/>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AB22" t="n">
         <v>0</v>
       </c>
@@ -3109,31 +3485,31 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Wind Engineering of High-Rise Buildings</t>
+          <t>White Paper MVRDV NEXT</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Book</t>
+          <t>White paper</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Committee-Driven</t>
+          <t>Program Partnership</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>916</t>
+          <t>905a</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>RD</t>
+          <t>WM</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -3143,13 +3519,13 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Commissioned Research</t>
+          <t>Program Partnership</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Internal idea</t>
+          <t>Obligatory sponsor deliverable</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -3159,40 +3535,72 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Committee</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>Wind Engineering Cmte</t>
-        </is>
-      </c>
+          <t>Client + RTL</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Commissioned Research</t>
-        </is>
-      </c>
-      <c r="O23" t="inlineStr"/>
+          <t>Program Partner</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>MVRDV NEXT (in-kind)</t>
+        </is>
+      </c>
       <c r="P23" t="n">
-        <v>40000</v>
+        <v>0</v>
       </c>
       <c r="Q23" t="n">
         <v>0</v>
       </c>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
-      <c r="T23" t="inlineStr"/>
-      <c r="U23" t="inlineStr"/>
-      <c r="V23" t="inlineStr"/>
-      <c r="W23" t="inlineStr"/>
-      <c r="X23" t="inlineStr"/>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
       <c r="Y23" t="inlineStr"/>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="AA23" t="inlineStr"/>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AB23" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Update: content_projects.xlsx [2026-04-14 22:13 UTC]
</commit_message>
<xml_diff>
--- a/content_projects.xlsx
+++ b/content_projects.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC23"/>
+  <dimension ref="A1:AC24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3522,7 +3522,11 @@
           <t>Program Partnership</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J23" t="inlineStr">
         <is>
           <t>Obligatory sponsor deliverable</t>
@@ -3538,7 +3542,11 @@
           <t>Client + RTL</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N23" t="inlineStr">
         <is>
           <t>Program Partner</t>
@@ -3590,7 +3598,11 @@
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="Y23" t="inlineStr"/>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="Z23" t="inlineStr">
         <is>
           <t>2026-09-01</t>
@@ -3605,6 +3617,101 @@
         <v>0</v>
       </c>
       <c r="AC23" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Outdoor Wind Comfort Regulation Guide</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Book</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Committee-Driven</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>916</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>RD</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Commissioned Research</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Internal idea</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Committee</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Wind Engineering Cmte</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Commissioned Research</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr"/>
+      <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr"/>
+      <c r="AB24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC24" t="inlineStr">
         <is>
           <t>Confirmed</t>
         </is>

</xml_diff>

<commit_message>
Update: content_projects.xlsx [2026-04-14 22:16 UTC]
</commit_message>
<xml_diff>
--- a/content_projects.xlsx
+++ b/content_projects.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC24"/>
+  <dimension ref="A1:AC25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3661,7 +3661,11 @@
           <t>Commissioned Research</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J24" t="inlineStr">
         <is>
           <t>Internal idea</t>
@@ -3687,33 +3691,192 @@
           <t>Commissioned Research</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="P24" t="n">
         <v>0</v>
       </c>
       <c r="Q24" t="n">
         <v>0</v>
       </c>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr"/>
-      <c r="U24" t="inlineStr"/>
-      <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr"/>
-      <c r="X24" t="inlineStr"/>
-      <c r="Y24" t="inlineStr"/>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="Z24" t="inlineStr">
         <is>
           <t>2026-12-31</t>
         </is>
       </c>
-      <c r="AA24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AB24" t="n">
         <v>0</v>
       </c>
       <c r="AC24" t="inlineStr">
         <is>
           <t>Confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Research Roadmap 2.0</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>PDF report</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Committee-Driven</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>704</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Internal idea</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>External Contributors</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="AA25" t="inlineStr"/>
+      <c r="AB25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>Pending</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update: content_projects.xlsx [2026-04-14 22:18 UTC]
</commit_message>
<xml_diff>
--- a/content_projects.xlsx
+++ b/content_projects.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC25"/>
+  <dimension ref="A1:AC26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3795,8 +3795,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="J25" t="inlineStr">
         <is>
           <t>Internal idea</t>
@@ -3812,13 +3820,21 @@
           <t>External Contributors</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="N25" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr"/>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="P25" t="n">
         <v>0</v>
       </c>
@@ -3870,11 +3886,138 @@
           <t>2026-09-21</t>
         </is>
       </c>
-      <c r="AA25" t="inlineStr"/>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
       <c r="AB25" t="n">
         <v>0</v>
       </c>
       <c r="AC25" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>RFR China Façade Book</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Book</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Other Sponsorship</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>705</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Commissioned Research</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Internal commitment</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Print</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Other CVU Team</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Commissioned Research</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>Unlikely to happen</t>
+        </is>
+      </c>
+      <c r="AB26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC26" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>

</xml_diff>

<commit_message>
Update: content_projects.xlsx [2026-04-14 22:19 UTC]
</commit_message>
<xml_diff>
--- a/content_projects.xlsx
+++ b/content_projects.xlsx
@@ -3485,16 +3485,16 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Outdoor Wind Comfort Regulation Guide</t>
+          <t>Research Roadmap 2.0</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Book</t>
+          <t>PDF report</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -3504,22 +3504,22 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>916</t>
+          <t>704</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>RD</t>
+          <t>DS</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Commissioned Research</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -3534,22 +3534,22 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Committee</t>
+          <t>External Contributors</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Wind Engineering Cmte</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Commissioned Research</t>
+          <t>None</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -3565,47 +3565,47 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>2026-12-31</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="AA23" t="inlineStr">
@@ -3618,32 +3618,32 @@
       </c>
       <c r="AC23" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Research Roadmap 2.0</t>
+          <t>RFR China Façade Book</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>PDF report</t>
+          <t>Book</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Committee-Driven</t>
+          <t>Other Sponsorship</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>704</t>
+          <t>705</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -3653,12 +3653,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Commissioned Research</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -3668,17 +3668,17 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Internal idea</t>
+          <t>Internal commitment</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Print</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>External Contributors</t>
+          <t>Other CVU Team</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -3688,7 +3688,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Commissioned Research</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -3704,32 +3704,32 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="X24" t="inlineStr">
@@ -3739,17 +3739,17 @@
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Unlikely to happen</t>
         </is>
       </c>
       <c r="AB24" t="n">
@@ -3763,11 +3763,11 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>RFR China Façade Book</t>
+          <t>Wind Engineering of High-Rise Buildings</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3777,17 +3777,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Other Sponsorship</t>
+          <t>Committee-Driven</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>705</t>
+          <t>916</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>DS</t>
+          <t>RD</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -3807,22 +3807,22 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Internal commitment</t>
+          <t>Internal idea</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Print</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Other CVU Team</t>
+          <t>Committee</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Wind Engineering Cmte</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -3836,59 +3836,59 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>0</v>
+        <v>40000</v>
       </c>
       <c r="Q25" t="n">
         <v>0</v>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="X25" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>Unlikely to happen</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="AB25" t="n">
@@ -3902,11 +3902,11 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Wind Engineering of High-Rise Buildings</t>
+          <t>Outdoor Wind Comfort Regulation Guide</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3967,7 +3967,7 @@
       </c>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="n">
-        <v>40000</v>
+        <v>0</v>
       </c>
       <c r="Q26" t="n">
         <v>0</v>
@@ -3982,7 +3982,7 @@
       <c r="Y26" t="inlineStr"/>
       <c r="Z26" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="AA26" t="inlineStr">

</xml_diff>